<commit_message>
Updated Facility Type for P2 and P5 to common
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wmollel\Documents\MEET2\input\Studies\C3\C3_Prototypical_Sites\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wmollel\Documents\MAES\input\Studies\C3\C3_Prototypical_Sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A316282E-9CD7-4B15-B2B3-0D72DC366A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B8F390-CA4F-4BF0-97FB-A2206E1A0E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -580,13 +580,13 @@
     <t>Max Downstream Equipment Capacity [scfh]</t>
   </si>
   <si>
-    <t>Production</t>
-  </si>
-  <si>
     <t>Gas</t>
   </si>
   <si>
     <t xml:space="preserve">Gas </t>
+  </si>
+  <si>
+    <t>Common</t>
   </si>
 </sst>
 </file>
@@ -1238,7 +1238,7 @@
         <v>120</v>
       </c>
       <c r="B6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -1392,7 +1392,7 @@
         <v>83</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E2" t="s">
         <v>16</v>
@@ -1490,7 +1490,7 @@
         <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
@@ -3896,7 +3896,7 @@
         <v>20</v>
       </c>
       <c r="O2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="P2" t="s">
         <v>34</v>
@@ -3998,7 +3998,7 @@
         <v>5.9867000000000002E-3</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G2" s="3">
         <v>0.75</v>
@@ -4058,7 +4058,7 @@
         <v>5.9867000000000002E-3</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G4" s="3">
         <v>1</v>
@@ -4620,7 +4620,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G2" t="s">
         <v>107</v>

</xml_diff>

<commit_message>
minor fix for using ccee flag
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wmollel\Documents\MAES\input\Studies\C3\C3_Prototypical_Sites\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES2\input\Studies\C3\C3_Prototypical_Sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B8F390-CA4F-4BF0-97FB-A2206E1A0E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25569D77-CF6E-489B-BA54-98D3BAD06FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="894" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="180">
   <si>
     <t>Simulation Start Date</t>
   </si>
@@ -460,9 +460,6 @@
     <t>water_gas_sales</t>
   </si>
   <si>
-    <t>Heaters</t>
-  </si>
-  <si>
     <t>Number of Pneumatics</t>
   </si>
   <si>
@@ -587,6 +584,9 @@
   </si>
   <si>
     <t>Common</t>
+  </si>
+  <si>
+    <t>Tank Controlled [True, False]</t>
   </si>
 </sst>
 </file>
@@ -787,7 +787,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -889,6 +889,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -1220,7 +1221,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>32</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1238,7 +1239,7 @@
         <v>120</v>
       </c>
       <c r="B6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -1249,7 +1250,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:AF3"/>
+  <dimension ref="A1:AG3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -1278,12 +1279,13 @@
     <col min="28" max="28" width="18.85546875" customWidth="1"/>
     <col min="29" max="29" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="63.7109375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="14" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.5703125" customWidth="1"/>
+    <col min="32" max="32" width="63.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="9" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" s="9" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -1357,31 +1359,34 @@
         <v>128</v>
       </c>
       <c r="Y1" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="Z1" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="Z1" s="20" t="s">
+      <c r="AA1" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="AA1" s="20" t="s">
+      <c r="AB1" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="AB1" s="20" t="s">
+      <c r="AC1" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="AC1" s="20" t="s">
+      <c r="AD1" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="AD1" s="20" t="s">
-        <v>176</v>
-      </c>
-      <c r="AE1" s="8" t="s">
+      <c r="AE1" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="AF1" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="AF1" s="8" t="s">
+      <c r="AG1" s="8" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -1392,7 +1397,7 @@
         <v>83</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E2" t="s">
         <v>16</v>
@@ -1472,14 +1477,17 @@
       <c r="AD2" s="27">
         <v>5000</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AE2" s="41" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF2" t="s">
         <v>113</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -1490,7 +1498,7 @@
         <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
@@ -1570,10 +1578,13 @@
       <c r="AD3" s="27">
         <v>5000</v>
       </c>
-      <c r="AE3" t="s">
+      <c r="AE3" s="41" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF3" t="s">
         <v>112</v>
       </c>
-      <c r="AF3" t="s">
+      <c r="AG3" t="s">
         <v>117</v>
       </c>
     </row>
@@ -1605,7 +1616,7 @@
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1613,13 +1624,13 @@
         <v>69</v>
       </c>
       <c r="B2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C2" t="s">
         <v>153</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>154</v>
-      </c>
-      <c r="D2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1627,13 +1638,13 @@
         <v>69</v>
       </c>
       <c r="B3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" t="s">
         <v>156</v>
-      </c>
-      <c r="C3" t="s">
-        <v>154</v>
-      </c>
-      <c r="D3" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1641,13 +1652,13 @@
         <v>69</v>
       </c>
       <c r="B5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" t="s">
         <v>158</v>
-      </c>
-      <c r="C5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D5" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1655,13 +1666,13 @@
         <v>69</v>
       </c>
       <c r="B6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" t="s">
         <v>160</v>
-      </c>
-      <c r="C6" t="s">
-        <v>154</v>
-      </c>
-      <c r="D6" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1669,13 +1680,13 @@
         <v>69</v>
       </c>
       <c r="B7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D7" t="s">
         <v>162</v>
-      </c>
-      <c r="C7" t="s">
-        <v>154</v>
-      </c>
-      <c r="D7" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1683,13 +1694,13 @@
         <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1697,13 +1708,13 @@
         <v>69</v>
       </c>
       <c r="B10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -1713,7 +1724,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F101BBB2-448E-4A39-BC60-8556E9F30D1D}">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
@@ -1803,7 +1814,7 @@
         <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="F5" t="s">
         <v>38</v>
@@ -1826,7 +1837,7 @@
         <v>69</v>
       </c>
       <c r="E6" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
         <v>39</v>
@@ -1849,7 +1860,7 @@
         <v>69</v>
       </c>
       <c r="E7" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="F7" t="s">
         <v>62</v>
@@ -1872,7 +1883,7 @@
         <v>69</v>
       </c>
       <c r="E8" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="F8" t="s">
         <v>62</v>
@@ -1881,29 +1892,6 @@
         <v>87</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" t="s">
-        <v>134</v>
-      </c>
-      <c r="F9" t="s">
-        <v>62</v>
-      </c>
-      <c r="G9" t="s">
-        <v>135</v>
-      </c>
-    </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>43</v>
@@ -1918,13 +1906,13 @@
         <v>69</v>
       </c>
       <c r="E10" t="s">
-        <v>134</v>
+        <v>83</v>
       </c>
       <c r="F10" t="s">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="G10" t="s">
-        <v>136</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1935,13 +1923,13 @@
         <v>69</v>
       </c>
       <c r="C12" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
         <v>69</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F12" t="s">
         <v>38</v>
@@ -1958,19 +1946,19 @@
         <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
         <v>69</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F13" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="G13" t="s">
-        <v>40</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1981,42 +1969,42 @@
         <v>69</v>
       </c>
       <c r="C14" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
         <v>69</v>
       </c>
       <c r="E14" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F14" t="s">
         <v>62</v>
       </c>
       <c r="G14" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C15" t="s">
-        <v>134</v>
-      </c>
-      <c r="D15" t="s">
-        <v>69</v>
-      </c>
-      <c r="E15" t="s">
-        <v>32</v>
-      </c>
-      <c r="F15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" t="s">
+        <v>67</v>
+      </c>
+      <c r="F16" t="s">
         <v>62</v>
       </c>
-      <c r="G15" t="s">
-        <v>87</v>
+      <c r="G16" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2027,198 +2015,83 @@
         <v>69</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D17" t="s">
         <v>69</v>
       </c>
       <c r="E17" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="F17" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="G17" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" t="s">
-        <v>69</v>
-      </c>
-      <c r="C19" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19" t="s">
-        <v>22</v>
-      </c>
-      <c r="F19" t="s">
-        <v>38</v>
-      </c>
-      <c r="G19" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" t="s">
-        <v>69</v>
-      </c>
-      <c r="C20" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" t="s">
-        <v>69</v>
-      </c>
-      <c r="E20" t="s">
-        <v>22</v>
-      </c>
-      <c r="F20" t="s">
-        <v>62</v>
-      </c>
-      <c r="G20" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>43</v>
-      </c>
-      <c r="B21" t="s">
-        <v>69</v>
-      </c>
-      <c r="C21" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" t="s">
-        <v>69</v>
-      </c>
-      <c r="E21" t="s">
-        <v>22</v>
-      </c>
-      <c r="F21" t="s">
-        <v>62</v>
-      </c>
-      <c r="G21" t="s">
-        <v>87</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>43</v>
-      </c>
-      <c r="B23" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" t="s">
-        <v>22</v>
-      </c>
-      <c r="D23" t="s">
-        <v>69</v>
-      </c>
-      <c r="E23" t="s">
-        <v>67</v>
-      </c>
-      <c r="F23" t="s">
-        <v>62</v>
-      </c>
-      <c r="G23" t="s">
-        <v>88</v>
-      </c>
+      <c r="A23" s="35"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="35"/>
+      <c r="G23" s="35"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>43</v>
-      </c>
-      <c r="B24" t="s">
-        <v>69</v>
-      </c>
-      <c r="C24" t="s">
-        <v>22</v>
-      </c>
-      <c r="D24" t="s">
-        <v>69</v>
-      </c>
-      <c r="E24" t="s">
-        <v>67</v>
-      </c>
-      <c r="F24" t="s">
-        <v>62</v>
-      </c>
-      <c r="G24" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="35"/>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="35"/>
-      <c r="G30" s="35"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="35"/>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="35"/>
-      <c r="B32" s="35"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="35"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="35"/>
-      <c r="B33" s="35"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="35"/>
-      <c r="B34" s="35"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
-      <c r="G34" s="35"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="35"/>
-      <c r="B35" s="35"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="35"/>
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
-      <c r="G35" s="35"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="35"/>
-      <c r="B36" s="35"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="35"/>
-      <c r="F36" s="35"/>
-      <c r="G36" s="35"/>
+      <c r="A24" s="35"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="35"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="35"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="35"/>
+      <c r="G25" s="35"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="35"/>
+      <c r="B26" s="35"/>
+      <c r="C26" s="35"/>
+      <c r="D26" s="35"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="35"/>
+      <c r="G26" s="35"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="35"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="35"/>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="35"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="35"/>
+      <c r="B29" s="35"/>
+      <c r="C29" s="35"/>
+      <c r="D29" s="35"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="35"/>
+      <c r="G29" s="35"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2455,7 +2328,7 @@
         <v>69</v>
       </c>
       <c r="E12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F12" t="s">
         <v>38</v>
@@ -2478,7 +2351,7 @@
         <v>69</v>
       </c>
       <c r="E13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F13" t="s">
         <v>39</v>
@@ -2501,7 +2374,7 @@
         <v>69</v>
       </c>
       <c r="E14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F14" t="s">
         <v>62</v>
@@ -2524,7 +2397,7 @@
         <v>69</v>
       </c>
       <c r="E15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F15" t="s">
         <v>62</v>
@@ -2541,7 +2414,7 @@
         <v>69</v>
       </c>
       <c r="C17" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D17" t="s">
         <v>69</v>
@@ -2564,7 +2437,7 @@
         <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D18" t="s">
         <v>69</v>
@@ -2587,7 +2460,7 @@
         <v>69</v>
       </c>
       <c r="C19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D19" t="s">
         <v>69</v>
@@ -2610,7 +2483,7 @@
         <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D20" t="s">
         <v>69</v>
@@ -2694,7 +2567,7 @@
         <v>62</v>
       </c>
       <c r="G24" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -2734,7 +2607,7 @@
         <v>69</v>
       </c>
       <c r="E28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F28" t="s">
         <v>38</v>
@@ -2754,7 +2627,7 @@
         <v>69</v>
       </c>
       <c r="E29" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F29" t="s">
         <v>39</v>
@@ -2774,7 +2647,7 @@
         <v>69</v>
       </c>
       <c r="E31" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F31" t="s">
         <v>39</v>
@@ -2797,7 +2670,7 @@
         <v>69</v>
       </c>
       <c r="E33" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F33" t="s">
         <v>38</v>
@@ -2820,7 +2693,7 @@
         <v>69</v>
       </c>
       <c r="E34" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F34" t="s">
         <v>62</v>
@@ -2843,7 +2716,7 @@
         <v>69</v>
       </c>
       <c r="E36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F36" t="s">
         <v>38</v>
@@ -2866,7 +2739,7 @@
         <v>69</v>
       </c>
       <c r="E37" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F37" t="s">
         <v>62</v>
@@ -3119,7 +2992,7 @@
         <v>69</v>
       </c>
       <c r="E12" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F12" t="s">
         <v>38</v>
@@ -3142,7 +3015,7 @@
         <v>69</v>
       </c>
       <c r="E13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F13" t="s">
         <v>39</v>
@@ -3165,7 +3038,7 @@
         <v>69</v>
       </c>
       <c r="E14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F14" t="s">
         <v>62</v>
@@ -3188,7 +3061,7 @@
         <v>69</v>
       </c>
       <c r="E15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F15" t="s">
         <v>62</v>
@@ -3211,7 +3084,7 @@
         <v>69</v>
       </c>
       <c r="E17" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F17" t="s">
         <v>38</v>
@@ -3234,7 +3107,7 @@
         <v>69</v>
       </c>
       <c r="E18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F18" t="s">
         <v>39</v>
@@ -3257,7 +3130,7 @@
         <v>69</v>
       </c>
       <c r="E19" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F19" t="s">
         <v>62</v>
@@ -3280,7 +3153,7 @@
         <v>69</v>
       </c>
       <c r="E20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F20" t="s">
         <v>62</v>
@@ -3297,7 +3170,7 @@
         <v>69</v>
       </c>
       <c r="C22" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D22" t="s">
         <v>69</v>
@@ -3320,7 +3193,7 @@
         <v>69</v>
       </c>
       <c r="C23" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D23" t="s">
         <v>69</v>
@@ -3343,7 +3216,7 @@
         <v>69</v>
       </c>
       <c r="C24" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D24" t="s">
         <v>69</v>
@@ -3366,7 +3239,7 @@
         <v>69</v>
       </c>
       <c r="C25" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D25" t="s">
         <v>69</v>
@@ -3392,7 +3265,7 @@
         <v>69</v>
       </c>
       <c r="C27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D27" t="s">
         <v>69</v>
@@ -3415,7 +3288,7 @@
         <v>69</v>
       </c>
       <c r="C28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D28" t="s">
         <v>69</v>
@@ -3438,7 +3311,7 @@
         <v>69</v>
       </c>
       <c r="C29" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D29" t="s">
         <v>69</v>
@@ -3461,7 +3334,7 @@
         <v>69</v>
       </c>
       <c r="C30" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D30" t="s">
         <v>69</v>
@@ -3568,7 +3441,7 @@
         <v>62</v>
       </c>
       <c r="G36" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -3614,7 +3487,7 @@
         <v>62</v>
       </c>
       <c r="G39" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -3635,7 +3508,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
@@ -3675,10 +3548,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>137</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>137</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3699,18 +3572,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -3896,7 +3761,7 @@
         <v>20</v>
       </c>
       <c r="O2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="P2" t="s">
         <v>34</v>
@@ -3998,7 +3863,7 @@
         <v>5.9867000000000002E-3</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G2" s="3">
         <v>0.75</v>
@@ -4058,7 +3923,7 @@
         <v>5.9867000000000002E-3</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G4" s="3">
         <v>1</v>
@@ -4223,16 +4088,16 @@
         <v>8</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E1" s="39" t="s">
+        <v>142</v>
+      </c>
+      <c r="F1" s="39" t="s">
         <v>143</v>
       </c>
-      <c r="F1" s="39" t="s">
+      <c r="G1" s="39" t="s">
         <v>144</v>
-      </c>
-      <c r="G1" s="39" t="s">
-        <v>145</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>61</v>
@@ -4246,10 +4111,10 @@
         <v>69</v>
       </c>
       <c r="B2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C2" t="s">
         <v>149</v>
-      </c>
-      <c r="C2" t="s">
-        <v>150</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -4264,7 +4129,7 @@
         <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I2" t="s">
         <v>92</v>
@@ -4303,28 +4168,28 @@
         <v>8</v>
       </c>
       <c r="D1" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="33" t="s">
         <v>138</v>
       </c>
-      <c r="E1" s="33" t="s">
+      <c r="F1" s="33" t="s">
         <v>139</v>
       </c>
-      <c r="F1" s="33" t="s">
+      <c r="G1" s="31" t="s">
         <v>140</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="H1" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="I1" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="J1" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="K1" s="24" t="s">
         <v>144</v>
-      </c>
-      <c r="K1" s="24" t="s">
-        <v>145</v>
       </c>
       <c r="L1" s="8" t="s">
         <v>61</v>
@@ -4338,10 +4203,10 @@
         <v>69</v>
       </c>
       <c r="B2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" t="s">
         <v>146</v>
-      </c>
-      <c r="C2" t="s">
-        <v>147</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -4368,7 +4233,7 @@
         <v>20</v>
       </c>
       <c r="L2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="M2" t="s">
         <v>92</v>
@@ -4620,7 +4485,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G2" t="s">
         <v>107</v>

</xml_diff>

<commit_message>
added timseries and pdf code
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES2\input\Studies\C3\C3_Prototypical_Sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25569D77-CF6E-489B-BA54-98D3BAD06FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD30D2E-66A2-46F9-88AA-572643CAD6A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="894" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25070" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="894" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -1466,16 +1466,16 @@
         <v>2</v>
       </c>
       <c r="AA2" s="22">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="AB2" s="27">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="AC2" s="27">
         <v>10000</v>
       </c>
       <c r="AD2" s="27">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="AE2" s="41" t="b">
         <v>1</v>
@@ -1567,16 +1567,16 @@
         <v>2</v>
       </c>
       <c r="AA3" s="22">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="AB3" s="27">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="AC3" s="27">
         <v>10000</v>
       </c>
       <c r="AD3" s="27">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="AE3" s="41" t="b">
         <v>1</v>
@@ -3872,7 +3872,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="16">
-        <v>0.01</v>
+        <v>0.5</v>
       </c>
       <c r="J2" s="16">
         <v>1</v>
@@ -3932,7 +3932,7 @@
         <v>1</v>
       </c>
       <c r="I4" s="16">
-        <v>0.01</v>
+        <v>0.5</v>
       </c>
       <c r="J4" s="16">
         <v>1</v>

</xml_diff>

<commit_message>
tank battery fix to get random initial state duration for thief hatch mechansitic
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES2\input\Studies\C3\C3_Prototypical_Sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0FC4C93-B6B7-4177-980B-35BB37D91AAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34971A79-A700-4A42-9ECC-F142D1C506A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25040" yWindow="-80" windowWidth="25120" windowHeight="16080" tabRatio="894" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25070" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="894" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -1215,7 +1215,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1396,7 +1396,7 @@
         <v>365</v>
       </c>
       <c r="I2" s="7">
-        <v>4.3276E-3</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1444,22 +1444,22 @@
         <v>0.14960999999999999</v>
       </c>
       <c r="Y2" s="22">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="Z2" s="22">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="AA2" s="22">
-        <v>0.01</v>
+        <v>0.06</v>
       </c>
       <c r="AB2" s="27">
-        <v>6000</v>
+        <v>18000</v>
       </c>
       <c r="AC2" s="27">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="AD2" s="27">
-        <v>7000</v>
+        <v>19000</v>
       </c>
       <c r="AE2" s="41" t="b">
         <v>1</v>
@@ -1497,7 +1497,7 @@
         <v>365</v>
       </c>
       <c r="I3" s="7">
-        <v>4.3276E-3</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -1545,22 +1545,22 @@
         <v>0.14960999999999999</v>
       </c>
       <c r="Y3" s="22">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="Z3" s="22">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="AA3" s="22">
-        <v>0.01</v>
+        <v>0.06</v>
       </c>
       <c r="AB3" s="27">
-        <v>6000</v>
+        <v>18000</v>
       </c>
       <c r="AC3" s="27">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="AD3" s="27">
-        <v>7000</v>
+        <v>19000</v>
       </c>
       <c r="AE3" s="41" t="b">
         <v>1</v>
@@ -1942,7 +1942,7 @@
         <v>61</v>
       </c>
       <c r="G13" t="s">
-        <v>85</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1965,7 +1965,7 @@
         <v>61</v>
       </c>
       <c r="G14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -3856,7 +3856,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="16">
-        <v>1E-3</v>
+        <v>0.05</v>
       </c>
       <c r="J2" s="16">
         <v>1</v>
@@ -3916,7 +3916,7 @@
         <v>1</v>
       </c>
       <c r="I4" s="16">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="J4" s="16">
         <v>1</v>

</xml_diff>

<commit_message>
updated tanks model for controlled and uncontrolled modes. UPDATE TANK STUDY SHEET FROM TEMPLATE.
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES2\input\Studies\C3\C3_Prototypical_Sites\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES_dev\input\Studies\C3\C3_Prototypical_Sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4C88CB3-214D-43C2-ABD1-047773863BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B476F719-337F-48C9-A5ED-C455AA4C123F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25070" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="894" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="894" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -1188,13 +1188,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>118</v>
       </c>
@@ -1235,41 +1235,41 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:AG3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="31.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.81640625" bestFit="1" customWidth="1"/>
     <col min="17" max="18" width="12" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="18.453125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="21" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.5703125" customWidth="1"/>
-    <col min="26" max="26" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="18.85546875" customWidth="1"/>
-    <col min="29" max="29" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.5703125" customWidth="1"/>
-    <col min="32" max="32" width="63.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.54296875" customWidth="1"/>
+    <col min="26" max="26" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.81640625" customWidth="1"/>
+    <col min="29" max="29" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.54296875" customWidth="1"/>
+    <col min="32" max="32" width="63.7265625" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="14" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="9" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" s="9" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1471,7 +1471,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -1581,15 +1581,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ED1D13E-94B9-4C06-8746-12064F7C9C36}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>68</v>
       </c>
@@ -1645,7 +1645,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>68</v>
       </c>
@@ -1659,7 +1659,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>68</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>68</v>
       </c>
@@ -1687,7 +1687,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>68</v>
       </c>
@@ -1709,18 +1709,18 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F101BBB2-448E-4A39-BC60-8556E9F30D1D}">
   <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1807,7 +1807,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1830,7 +1830,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -1853,7 +1853,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -1945,7 +1945,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>43</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="35"/>
       <c r="B23" s="35"/>
       <c r="C23" s="35"/>
@@ -2023,7 +2023,7 @@
       <c r="F23" s="35"/>
       <c r="G23" s="35"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="35"/>
       <c r="B24" s="35"/>
       <c r="C24" s="35"/>
@@ -2032,7 +2032,7 @@
       <c r="F24" s="35"/>
       <c r="G24" s="35"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="35"/>
       <c r="B25" s="35"/>
       <c r="C25" s="35"/>
@@ -2041,7 +2041,7 @@
       <c r="F25" s="35"/>
       <c r="G25" s="35"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="35"/>
       <c r="B26" s="35"/>
       <c r="C26" s="35"/>
@@ -2050,7 +2050,7 @@
       <c r="F26" s="35"/>
       <c r="G26" s="35"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="35"/>
       <c r="B27" s="35"/>
       <c r="C27" s="35"/>
@@ -2059,7 +2059,7 @@
       <c r="F27" s="35"/>
       <c r="G27" s="35"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="35"/>
       <c r="B28" s="35"/>
       <c r="C28" s="35"/>
@@ -2068,7 +2068,7 @@
       <c r="F28" s="35"/>
       <c r="G28" s="35"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="35"/>
       <c r="B29" s="35"/>
       <c r="C29" s="35"/>
@@ -2085,18 +2085,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26CFFBB7-31C2-4A1A-B76F-A7AE02F8A8A9}">
   <dimension ref="A1:G38"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -2183,7 +2183,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>43</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -2482,10 +2482,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="E21" s="25"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>43</v>
       </c>
@@ -2531,7 +2531,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -2577,7 +2577,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -2597,7 +2597,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -2617,7 +2617,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>43</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>43</v>
       </c>
@@ -2663,7 +2663,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -2732,7 +2732,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="35"/>
       <c r="B38" s="35"/>
       <c r="C38" s="35"/>
@@ -2749,18 +2749,18 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09131FE7-5CF0-4155-B869-9951A97BC4D6}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -2783,7 +2783,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -2916,7 +2916,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -2939,7 +2939,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -2985,7 +2985,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -3031,7 +3031,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -3054,7 +3054,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>43</v>
       </c>
@@ -3100,7 +3100,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>43</v>
       </c>
@@ -3192,7 +3192,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>43</v>
       </c>
@@ -3238,10 +3238,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="E26" s="25"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>43</v>
       </c>
@@ -3264,7 +3264,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>43</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>43</v>
       </c>
@@ -3356,10 +3356,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="E33" s="25"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>43</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -3474,7 +3474,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="35"/>
       <c r="B52" s="35"/>
       <c r="C52" s="35"/>
@@ -3493,12 +3493,12 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="20.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -3506,7 +3506,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>88</v>
       </c>
@@ -3530,7 +3530,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>62</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -3570,16 +3570,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" customWidth="1"/>
-    <col min="2" max="2" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.81640625" customWidth="1"/>
+    <col min="2" max="2" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7265625" customWidth="1"/>
     <col min="4" max="4" width="64" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -3596,7 +3596,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -3621,28 +3621,28 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D73FC3-98E2-4799-8AF9-F22493DEB849}">
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.81640625" customWidth="1"/>
+    <col min="8" max="8" width="11.7265625" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.54296875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="64" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="36" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="36" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A1" s="36" t="s">
         <v>4</v>
       </c>
@@ -3701,7 +3701,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -3768,18 +3768,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:Q4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="13" width="15.7109375" style="3" customWidth="1"/>
-    <col min="14" max="14" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="47.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" customWidth="1"/>
-    <col min="17" max="17" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="5" width="15.7265625" customWidth="1"/>
+    <col min="6" max="13" width="15.7265625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="47.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.7265625" customWidth="1"/>
+    <col min="17" max="17" width="17.7265625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="Q1" s="23"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -3880,7 +3880,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="F3"/>
       <c r="G3"/>
       <c r="H3"/>
@@ -3890,7 +3890,7 @@
       <c r="L3"/>
       <c r="M3"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>68</v>
       </c>
@@ -3950,9 +3950,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54F32634-6A66-440D-87B9-BD63D4037634}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4048,20 +4048,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E555FE-0E09-4108-A751-03C57701E3B2}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" customWidth="1"/>
+    <col min="6" max="6" width="22.26953125" customWidth="1"/>
+    <col min="7" max="7" width="17.81640625" customWidth="1"/>
+    <col min="8" max="8" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -4090,7 +4090,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4127,21 +4127,21 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4A5CC92-4603-445D-B55F-A91A4D1C2C13}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="6" width="12.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" customWidth="1"/>
+    <col min="5" max="6" width="12.7265625" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="58" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -4182,7 +4182,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4231,18 +4231,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A904CBC9-E240-4A6F-BB4B-8DAB1536C2C9}">
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="12.28515625" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" customWidth="1"/>
-    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="63.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" customWidth="1"/>
+    <col min="6" max="6" width="10.26953125" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="63.7265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
@@ -4301,7 +4301,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4368,26 +4368,26 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:U12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.85546875" customWidth="1"/>
-    <col min="11" max="12" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.81640625" customWidth="1"/>
+    <col min="11" max="12" width="26.453125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="9" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" s="9" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4517,34 +4517,34 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F3"/>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F4"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F5"/>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F6"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F7"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F8"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F9"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F10"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F11"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="F12"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tank Model update. Multi-setup for sep, tanks, probes and compressors. Check doc with Prajay.
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES_dev\input\Studies\C3\C3_Prototypical_Sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B476F719-337F-48C9-A5ED-C455AA4C123F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D5CF23-C6AD-49AC-B682-5427D226997A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="894" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="894" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -562,9 +562,6 @@
     <t>Mechanistic Thief Hatch pLeak</t>
   </si>
   <si>
-    <t>PRV Threshold [scfh]</t>
-  </si>
-  <si>
     <t>Tank Inlet Flow at Max Downstream Equipment Capacity</t>
   </si>
   <si>
@@ -581,6 +578,9 @@
   </si>
   <si>
     <t>Tank Controlled [True, False]</t>
+  </si>
+  <si>
+    <t>Overpressure Threshold [scfh]</t>
   </si>
 </sst>
 </file>
@@ -1188,13 +1188,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1210,20 +1210,20 @@
         <v>365</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>118</v>
       </c>
       <c r="B4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -1235,41 +1235,41 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:AG3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="31.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="18" width="12" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="21" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.54296875" customWidth="1"/>
-    <col min="26" max="26" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="18.81640625" customWidth="1"/>
-    <col min="29" max="29" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.54296875" customWidth="1"/>
-    <col min="32" max="32" width="63.7265625" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.5703125" customWidth="1"/>
+    <col min="26" max="26" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="18.85546875" customWidth="1"/>
+    <col min="29" max="29" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.5703125" customWidth="1"/>
+    <col min="32" max="32" width="63.7109375" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="14" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="9" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" s="9" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -1352,16 +1352,16 @@
         <v>170</v>
       </c>
       <c r="AB1" s="20" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC1" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="AC1" s="20" t="s">
+      <c r="AD1" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="AD1" s="20" t="s">
-        <v>173</v>
-      </c>
       <c r="AE1" s="39" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AF1" s="8" t="s">
         <v>107</v>
@@ -1370,7 +1370,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1381,7 +1381,7 @@
         <v>82</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E2" t="s">
         <v>16</v>
@@ -1471,7 +1471,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
@@ -1581,15 +1581,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ED1D13E-94B9-4C06-8746-12064F7C9C36}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1617,7 +1617,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>68</v>
       </c>
@@ -1645,7 +1645,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>68</v>
       </c>
@@ -1659,7 +1659,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>68</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>68</v>
       </c>
@@ -1687,7 +1687,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>68</v>
       </c>
@@ -1709,18 +1709,18 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F101BBB2-448E-4A39-BC60-8556E9F30D1D}">
   <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -1807,7 +1807,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1830,7 +1830,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -1853,7 +1853,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -1945,7 +1945,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>43</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="35"/>
       <c r="B23" s="35"/>
       <c r="C23" s="35"/>
@@ -2023,7 +2023,7 @@
       <c r="F23" s="35"/>
       <c r="G23" s="35"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="35"/>
       <c r="B24" s="35"/>
       <c r="C24" s="35"/>
@@ -2032,7 +2032,7 @@
       <c r="F24" s="35"/>
       <c r="G24" s="35"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="35"/>
       <c r="B25" s="35"/>
       <c r="C25" s="35"/>
@@ -2041,7 +2041,7 @@
       <c r="F25" s="35"/>
       <c r="G25" s="35"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="35"/>
       <c r="B26" s="35"/>
       <c r="C26" s="35"/>
@@ -2050,7 +2050,7 @@
       <c r="F26" s="35"/>
       <c r="G26" s="35"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="35"/>
       <c r="B27" s="35"/>
       <c r="C27" s="35"/>
@@ -2059,7 +2059,7 @@
       <c r="F27" s="35"/>
       <c r="G27" s="35"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="35"/>
       <c r="B28" s="35"/>
       <c r="C28" s="35"/>
@@ -2068,7 +2068,7 @@
       <c r="F28" s="35"/>
       <c r="G28" s="35"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="35"/>
       <c r="B29" s="35"/>
       <c r="C29" s="35"/>
@@ -2085,18 +2085,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26CFFBB7-31C2-4A1A-B76F-A7AE02F8A8A9}">
   <dimension ref="A1:G38"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -2183,7 +2183,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>43</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -2482,10 +2482,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E21" s="25"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>43</v>
       </c>
@@ -2531,7 +2531,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -2577,7 +2577,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -2597,7 +2597,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -2617,7 +2617,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>43</v>
       </c>
@@ -2640,7 +2640,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>43</v>
       </c>
@@ -2663,7 +2663,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -2732,7 +2732,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="35"/>
       <c r="B38" s="35"/>
       <c r="C38" s="35"/>
@@ -2749,18 +2749,18 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09131FE7-5CF0-4155-B869-9951A97BC4D6}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -2783,7 +2783,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>43</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -2916,7 +2916,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -2939,7 +2939,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -2985,7 +2985,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -3031,7 +3031,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -3054,7 +3054,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>43</v>
       </c>
@@ -3100,7 +3100,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>43</v>
       </c>
@@ -3192,7 +3192,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>43</v>
       </c>
@@ -3238,10 +3238,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E26" s="25"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>43</v>
       </c>
@@ -3264,7 +3264,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>43</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>43</v>
       </c>
@@ -3356,10 +3356,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E33" s="25"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>43</v>
       </c>
@@ -3405,7 +3405,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -3474,7 +3474,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="35"/>
       <c r="B52" s="35"/>
       <c r="C52" s="35"/>
@@ -3493,12 +3493,12 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -3506,7 +3506,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>88</v>
       </c>
@@ -3530,7 +3530,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>62</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -3570,16 +3570,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.81640625" customWidth="1"/>
-    <col min="2" max="2" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7265625" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="2" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" customWidth="1"/>
     <col min="4" max="4" width="64" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -3596,7 +3596,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -3621,28 +3621,28 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D73FC3-98E2-4799-8AF9-F22493DEB849}">
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultColWidth="9.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.81640625" customWidth="1"/>
-    <col min="8" max="8" width="11.7265625" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="64" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="36" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" s="36" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="36" t="s">
         <v>4</v>
       </c>
@@ -3701,7 +3701,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>20</v>
       </c>
       <c r="O2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="P2" t="s">
         <v>34</v>
@@ -3768,18 +3768,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:Q4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="15.7265625" customWidth="1"/>
-    <col min="6" max="13" width="15.7265625" style="3" customWidth="1"/>
-    <col min="14" max="14" width="24.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="47.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.7265625" customWidth="1"/>
-    <col min="17" max="17" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="13" width="15.7109375" style="3" customWidth="1"/>
+    <col min="14" max="14" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="47.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" customWidth="1"/>
+    <col min="17" max="17" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="Q1" s="23"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -3847,7 +3847,7 @@
         <v>5.9867000000000002E-3</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G2" s="3">
         <v>0.75</v>
@@ -3880,7 +3880,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F3"/>
       <c r="G3"/>
       <c r="H3"/>
@@ -3890,7 +3890,7 @@
       <c r="L3"/>
       <c r="M3"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>68</v>
       </c>
@@ -3907,7 +3907,7 @@
         <v>5.9867000000000002E-3</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G4" s="3">
         <v>1</v>
@@ -3950,9 +3950,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54F32634-6A66-440D-87B9-BD63D4037634}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4048,20 +4048,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E555FE-0E09-4108-A751-03C57701E3B2}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.26953125" customWidth="1"/>
-    <col min="5" max="5" width="19.81640625" customWidth="1"/>
-    <col min="6" max="6" width="22.26953125" customWidth="1"/>
-    <col min="7" max="7" width="17.81640625" customWidth="1"/>
-    <col min="8" max="8" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -4090,7 +4090,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4127,21 +4127,21 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4A5CC92-4603-445D-B55F-A91A4D1C2C13}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="6" width="12.7265625" customWidth="1"/>
-    <col min="7" max="7" width="14.1796875" customWidth="1"/>
+    <col min="5" max="6" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="58" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -4182,7 +4182,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4231,18 +4231,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A904CBC9-E240-4A6F-BB4B-8DAB1536C2C9}">
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="12.26953125" customWidth="1"/>
-    <col min="6" max="6" width="10.26953125" customWidth="1"/>
-    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="63.7265625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="63.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
@@ -4301,7 +4301,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4368,26 +4368,26 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:U12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="8.54296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.81640625" customWidth="1"/>
-    <col min="11" max="12" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.85546875" customWidth="1"/>
+    <col min="11" max="12" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="9" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" s="9" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -4469,7 +4469,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G2" t="s">
         <v>106</v>
@@ -4517,34 +4517,34 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F3"/>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F4"/>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F5"/>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F6"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F7"/>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F8"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F9"/>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F10"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F11"/>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F12"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
putting tank emitters in emission events
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES_dev\input\Studies\C3\C3_Prototypical_Sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D5CF23-C6AD-49AC-B682-5427D226997A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC94C102-1DE1-4B8E-A823-CFE6F157A45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="894" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25070" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="894" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="176">
   <si>
     <t>Simulation Start Date</t>
   </si>
@@ -553,21 +553,6 @@
     <t>FFLinks1</t>
   </si>
   <si>
-    <t>Mechanistic Thief Hatch Leak MTTR min [days]</t>
-  </si>
-  <si>
-    <t>Mechanistic Thief Hatch Leak MTTR max [days]</t>
-  </si>
-  <si>
-    <t>Mechanistic Thief Hatch pLeak</t>
-  </si>
-  <si>
-    <t>Tank Inlet Flow at Max Downstream Equipment Capacity</t>
-  </si>
-  <si>
-    <t>Max Downstream Equipment Capacity [scfh]</t>
-  </si>
-  <si>
     <t>Gas</t>
   </si>
   <si>
@@ -581,6 +566,15 @@
   </si>
   <si>
     <t>Overpressure Threshold [scfh]</t>
+  </si>
+  <si>
+    <t>Mechanisitic Overpressure Vent Leaks MTTR min [days]</t>
+  </si>
+  <si>
+    <t>Mechanisitic Overpressure Vent Leaks MTTR max [days]</t>
+  </si>
+  <si>
+    <t>Mechanisitic Overpressure Vent Leaks pLeak</t>
   </si>
 </sst>
 </file>
@@ -1215,7 +1209,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1223,7 +1217,7 @@
         <v>118</v>
       </c>
       <c r="B4" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1234,7 +1228,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:AG3"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -1261,15 +1255,13 @@
     <col min="26" max="26" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="18.85546875" customWidth="1"/>
-    <col min="29" max="29" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.5703125" customWidth="1"/>
-    <col min="32" max="32" width="63.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="18.5703125" customWidth="1"/>
+    <col min="30" max="30" width="63.7109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="14" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="9" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" s="9" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>4</v>
       </c>
@@ -1343,34 +1335,28 @@
         <v>126</v>
       </c>
       <c r="Y1" s="20" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="Z1" s="20" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="AA1" s="20" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="AB1" s="20" t="s">
-        <v>177</v>
-      </c>
-      <c r="AC1" s="20" t="s">
+        <v>172</v>
+      </c>
+      <c r="AC1" s="39" t="s">
         <v>171</v>
       </c>
-      <c r="AD1" s="20" t="s">
-        <v>172</v>
-      </c>
-      <c r="AE1" s="39" t="s">
-        <v>176</v>
-      </c>
-      <c r="AF1" s="8" t="s">
+      <c r="AD1" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="AG1" s="8" t="s">
+      <c r="AE1" s="8" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1381,7 +1367,7 @@
         <v>82</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="E2" t="s">
         <v>16</v>
@@ -1453,25 +1439,19 @@
         <v>0.2</v>
       </c>
       <c r="AB2" s="27">
-        <v>18000</v>
-      </c>
-      <c r="AC2" s="27">
-        <v>20000</v>
-      </c>
-      <c r="AD2" s="27">
-        <v>19000</v>
-      </c>
-      <c r="AE2" s="41" t="b">
+        <v>15000</v>
+      </c>
+      <c r="AC2" s="41" t="b">
         <v>1</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AD2" t="s">
         <v>112</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AE2" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -1482,7 +1462,7 @@
         <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
@@ -1554,21 +1534,15 @@
         <v>0.2</v>
       </c>
       <c r="AB3" s="27">
-        <v>18000</v>
-      </c>
-      <c r="AC3" s="27">
-        <v>20000</v>
-      </c>
-      <c r="AD3" s="27">
-        <v>19000</v>
-      </c>
-      <c r="AE3" s="41" t="b">
+        <v>15000</v>
+      </c>
+      <c r="AC3" s="41" t="b">
         <v>1</v>
       </c>
-      <c r="AF3" t="s">
+      <c r="AD3" t="s">
         <v>111</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AE3" t="s">
         <v>116</v>
       </c>
     </row>
@@ -3745,7 +3719,7 @@
         <v>20</v>
       </c>
       <c r="O2" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="P2" t="s">
         <v>34</v>
@@ -3847,7 +3821,7 @@
         <v>5.9867000000000002E-3</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G2" s="3">
         <v>0.75</v>
@@ -3907,7 +3881,7 @@
         <v>5.9867000000000002E-3</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G4" s="3">
         <v>1</v>
@@ -4469,7 +4443,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="G2" t="s">
         <v>106</v>

</xml_diff>

<commit_message>
Fac update with ps number and operator columns
</commit_message>
<xml_diff>
--- a/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
+++ b/input/Studies/C3/C3_Prototypical_Sites/P2_2stages_flare.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES2\input\Studies\C3\C3_Prototypical_Sites\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\METEC\MAES_development\input\Studies\C3\C3_Prototypical_Sites\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4C88CB3-214D-43C2-ABD1-047773863BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C0F1F93-3540-4B1C-9232-785ADB1CACCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25070" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="894" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="894" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Simulation Parameters" sheetId="1" r:id="rId1"/>
@@ -1215,7 +1215,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>100</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>